<commit_message>
Incorporación anteecdentes de boleta de garantía
</commit_message>
<xml_diff>
--- a/1- BB.DD. ADMINISTRACIÓN DE CONVENIOS/BB.DD. ADMINISTRACIÓN DE CONVENIOS.xlsx
+++ b/1- BB.DD. ADMINISTRACIÓN DE CONVENIOS/BB.DD. ADMINISTRACIÓN DE CONVENIOS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\IPLACEX\Año 2\PRÁCTICA IPLACEX\1- BB.DD. ADMINISTRACIÓN DE CONVENIOS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{884115A7-BC04-4D75-9A2D-31D8BDD6AB44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B085A9F-B04E-4BAD-BCEB-72513D9C9F2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{18284660-3B24-4DA8-BF56-23B927E5D51D}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
   <si>
     <t>CENTRO FORMADOR</t>
   </si>
@@ -142,6 +142,18 @@
   </si>
   <si>
     <t>TOTAL CUPO MES TENM</t>
+  </si>
+  <si>
+    <t>MONTO BOLETA DE GARANTÍA</t>
+  </si>
+  <si>
+    <t>FECHA DE INICIO DE VIGENCIA DE BOLETA DE GARANTÍA</t>
+  </si>
+  <si>
+    <t>FECHA DE TÉRMINO DE VIGENCIA DE BOLETA DE GARANTÍA</t>
+  </si>
+  <si>
+    <t>ASEGURADOR BOLETA DE GARANTÍA</t>
   </si>
 </sst>
 </file>
@@ -501,7 +513,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B1BCA1B-B5BD-47E2-A086-F6F86BD42E69}">
-  <dimension ref="A1:AJ1"/>
+  <dimension ref="A1:AN1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.140625" bestFit="1" customWidth="1"/>
@@ -512,16 +524,16 @@
     <col min="6" max="6" width="26" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="27.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="30.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21" customWidth="1"/>
-    <col min="10" max="10" width="26.5703125" customWidth="1"/>
-    <col min="11" max="29" width="21" customWidth="1"/>
-    <col min="30" max="30" width="22.7109375" customWidth="1"/>
-    <col min="31" max="31" width="21" customWidth="1"/>
-    <col min="32" max="32" width="32.5703125" customWidth="1"/>
-    <col min="33" max="34" width="21" customWidth="1"/>
+    <col min="9" max="13" width="21" customWidth="1"/>
+    <col min="14" max="14" width="26.5703125" customWidth="1"/>
+    <col min="15" max="33" width="21" customWidth="1"/>
+    <col min="34" max="34" width="22.7109375" customWidth="1"/>
+    <col min="35" max="35" width="21" customWidth="1"/>
+    <col min="36" max="36" width="32.5703125" customWidth="1"/>
+    <col min="37" max="38" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -550,82 +562,94 @@
         <v>9</v>
       </c>
       <c r="J1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="N1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="R1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="S1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="T1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="U1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="V1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="W1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="X1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="Y1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="AA1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="AB1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="AC1" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="AD1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="AE1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="AB1" s="2" t="s">
+      <c r="AF1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="AC1" s="2" t="s">
+      <c r="AG1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="AD1" s="2" t="s">
+      <c r="AH1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="AE1" s="2" t="s">
+      <c r="AI1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="AF1" s="2" t="s">
+      <c r="AJ1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AG1" s="2" t="s">
+      <c r="AK1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="AH1" s="2"/>
-      <c r="AI1" t="s">
+      <c r="AL1" s="2"/>
+      <c r="AM1" t="s">
         <v>7</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AN1" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>